<commit_message>
changed password in data file
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/OpenCartTestData.xlsx
+++ b/src/test/resources/testData/OpenCartTestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
@@ -57,9 +57,6 @@
     <t>fName1</t>
   </si>
   <si>
-    <t>password123</t>
-  </si>
-  <si>
     <t>fName2</t>
   </si>
   <si>
@@ -70,6 +67,9 @@
   </si>
   <si>
     <t>lName3</t>
+  </si>
+  <si>
+    <t>Nal12345</t>
   </si>
 </sst>
 </file>
@@ -416,14 +416,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -457,10 +457,10 @@
         <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
@@ -468,19 +468,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -488,19 +488,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
@@ -510,10 +510,10 @@
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="amit@123"/>
     <hyperlink ref="E2" r:id="rId2" display="amit@123"/>
-    <hyperlink ref="E3" r:id="rId3" display="amit@123"/>
-    <hyperlink ref="E4" r:id="rId4" display="amit@123"/>
+    <hyperlink ref="D3" r:id="rId3" display="amit@123"/>
+    <hyperlink ref="E3" r:id="rId4" display="amit@123"/>
     <hyperlink ref="D4" r:id="rId5" display="amit@123"/>
-    <hyperlink ref="D3" r:id="rId6" display="amit@123"/>
+    <hyperlink ref="E4" r:id="rId6" display="amit@123"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId7"/>
@@ -523,7 +523,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -532,7 +532,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>